<commit_message>
Add FAQs page + assistant and Loan Against Mutual Funds landing page
- New /faqs drill-down page with retrieval-only assistant, corpus in src/data/faqs.ts feeding UI + JSON-LD
- New /loan-against-mutual-funds isolated campaign landing page
- Link FAQs in mega-nav (Get Help) and footer (Company)
- Update docs/pages.md inventory + regenerate page-metadata xlsx
- launch.json: enable autoPort on astro-verify

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shriram-page-metadata.xlsx
+++ b/shriram-page-metadata.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -688,37 +688,37 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Core &amp; Company</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Become a Partner Today | Shriram Financial Services</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Partner with Shriram Financial Services and earn by helping investors trade and invest. Explore our franchise and referral partner program.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>/become-a-partner</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="inlineStr">
-        <is>
-          <t>https://thisisshon.github.io/become-a-partner</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Open a Demat Account Online | Shriram Financial Services</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>One good call changes everything. Open a fully digital Demat account with Shriram Financial Services using just your mobile number - 100% paperless and SEBI-regulated.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>/open-demat-campaign1</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>https://thisisshon.github.io/open-demat-campaign1</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -733,27 +733,27 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Karnataka Bank Customers | Shriram Financial Services</t>
+          <t>Loan Against Mutual Funds | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Karnataka Bank customers can seamlessly open a trading &amp; demat account with Shriram Financial Services. Know the process here.</t>
+          <t>Get a Loan Against Mutual Funds for personal needs - pledge your holdings instead of selling. Interest from 10.5%* p.a., 100% paperless, from an RBI-regulated NBFC.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>/karnataka-bank-customers</t>
+          <t>/loan-against-mutual-funds</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/karnataka-bank-customers</t>
+          <t>https://thisisshon.github.io/loan-against-mutual-funds</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -768,22 +768,22 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Open A Demat Account | Shriram Financial Services</t>
+          <t>Become a Partner Today | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Open a fully digital Demat and trading account in minutes with Shriram Financial Services. Zero paperwork, SEBI-regulated and secure.</t>
+          <t>Partner with Shriram Financial Services and earn by helping investors trade and invest. Explore our franchise and referral partner program.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>/open-demat-account</t>
+          <t>/become-a-partner</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/open-demat-account</t>
+          <t>https://thisisshon.github.io/become-a-partner</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -803,22 +803,22 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Sitemap - All Pages | Shriram Financial Services</t>
+          <t>Karnataka Bank Customers | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Browse the full site structure of Shriram Financial Services, covering all products, research tools, calculators and about pages.</t>
+          <t>Karnataka Bank customers can seamlessly open a trading &amp; demat account with Shriram Financial Services. Know the process here.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>/sitemap</t>
+          <t>/karnataka-bank-customers</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/sitemap</t>
+          <t>https://thisisshon.github.io/karnataka-bank-customers</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -833,27 +833,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Products</t>
+          <t>Core &amp; Company</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Invest in Bonds &amp; Debentures | Shriram Financial Services</t>
+          <t>Open A Demat Account | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Invest in government and corporate bonds for stable, predictable fixed-income returns with lower risk, via Shriram Financial Services.</t>
+          <t>Open a fully digital Demat and trading account in minutes with Shriram Financial Services. Zero paperwork, SEBI-regulated and secure.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>/bonds</t>
+          <t>/open-demat-account</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/bonds</t>
+          <t>https://thisisshon.github.io/open-demat-account</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -868,27 +868,27 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Products</t>
+          <t>Core &amp; Company</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Commodity Trading - MCX | Shriram Financial Services</t>
+          <t>Sitemap - All Pages | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Trade gold, silver &amp; crude oil on MCX with live commodity prices, expert insights and secure execution with Shriram Financial Services</t>
+          <t>Browse the full site structure of Shriram Financial Services, covering all products, research tools, calculators and about pages.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>/commodities</t>
+          <t>/sitemap</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/commodities</t>
+          <t>https://thisisshon.github.io/sitemap</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -908,22 +908,22 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Currency Trading - Forex Pairs | Shriram Financial Services</t>
+          <t>Invest in Bonds &amp; Debentures | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Trade USD/INR, EUR/INR &amp; other currency pairs online with competitive spreads and real-time insights from Shriram Financial Services. Start today.</t>
+          <t>Invest in government and corporate bonds for stable, predictable fixed-income returns with lower risk, via Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>/currency</t>
+          <t>/bonds</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/currency</t>
+          <t>https://thisisshon.github.io/bonds</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -943,22 +943,22 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>F&amp;O Trading - Futures &amp; Options | Shriram Financial Services</t>
+          <t>Commodity Trading - MCX | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Trade futures &amp; options (F&amp;O) on NSE &amp; BSE at flat Rs 100/lot. SEBI-registered F&amp;O advisory and margin guidance from Shriram Financial Services.</t>
+          <t>Trade gold, silver &amp; crude oil on MCX with live commodity prices, expert insights and secure execution with Shriram Financial Services</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>/derivatives</t>
+          <t>/commodities</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/derivatives</t>
+          <t>https://thisisshon.github.io/commodities</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -978,22 +978,22 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Buy Equity Stocks - NSE &amp; BSE | Shriram Financial Services</t>
+          <t>Currency Trading - Forex Pairs | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Buy equity stocks online on NSE &amp; BSE with SEBI-registered research, real-time market data &amp; expert insights from Shriram Financial Services.</t>
+          <t>Trade USD/INR, EUR/INR &amp; other currency pairs online with competitive spreads and real-time insights from Shriram Financial Services. Start today.</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>/equity</t>
+          <t>/currency</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/equity</t>
+          <t>https://thisisshon.github.io/currency</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -1013,22 +1013,22 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>ETF Investing - Exchange Funds | Shriram Financial Services</t>
+          <t>F&amp;O Trading - Futures &amp; Options | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Diversify your portfolio with ETFs tracking indices, sectors &amp; commodities. Trade with low expense ratios via Shriram Financial Services.</t>
+          <t>Trade futures &amp; options (F&amp;O) on NSE &amp; BSE at flat Rs 100/lot. SEBI-registered F&amp;O advisory and margin guidance from Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>/etf</t>
+          <t>/derivatives</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/etf</t>
+          <t>https://thisisshon.github.io/derivatives</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1048,22 +1048,22 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Fixed Deposit - Up to 8.05%* p.a. | Shriram Financial Services</t>
+          <t>Buy Equity Stocks - NSE &amp; BSE | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Secure guaranteed returns of up to 8.05%* p.a. with fixed deposits from trusted partner institutions, offered by Shriram Financial Services.</t>
+          <t>Buy equity stocks online on NSE &amp; BSE with SEBI-registered research, real-time market data &amp; expert insights from Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>/fixed-deposit</t>
+          <t>/equity</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/fixed-deposit</t>
+          <t>https://thisisshon.github.io/equity</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -1083,22 +1083,22 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Invest in US Stocks &amp; ETFs | Shriram Financial Services</t>
+          <t>ETF Investing - Exchange Funds | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Access international markets and invest in top US stocks and global ETFs directly from your Indian account with Shriram Financial Services.</t>
+          <t>Diversify your portfolio with ETFs tracking indices, sectors &amp; commodities. Trade with low expense ratios via Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>/global-investing</t>
+          <t>/etf</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/global-investing</t>
+          <t>https://thisisshon.github.io/etf</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1118,22 +1118,22 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Apply for IPO - NSE &amp; BSE | Shriram Financial Services</t>
+          <t>Fixed Deposit - Up to 8.05%* p.a. | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Apply for the latest IPOs across NSE &amp; BSE and invest in companies as they debut on the stock market with Shriram Financial Services.</t>
+          <t>Secure guaranteed returns of up to 8.05%* p.a. with fixed deposits from trusted partner institutions, offered by Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>/ipo</t>
+          <t>/fixed-deposit</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/ipo</t>
+          <t>https://thisisshon.github.io/fixed-deposit</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -1153,22 +1153,22 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Loan Against Mutual Funds | Shriram Financial Services</t>
+          <t>Invest in US Stocks &amp; ETFs | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Get instant loans against your mutual fund holdings without redeeming investments. Quick, collateral-based LAMF from Shriram Financial Services.</t>
+          <t>Access international markets and invest in top US stocks and global ETFs directly from your Indian account with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>/loan-against-mutual-fund</t>
+          <t>/global-investing</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/loan-against-mutual-fund</t>
+          <t>https://thisisshon.github.io/global-investing</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1188,22 +1188,22 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Loan Against Shares (LAS) | Shriram Financial Services</t>
+          <t>Apply for IPO - NSE &amp; BSE | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Borrow against your equity portfolio at competitive interest rates while your shares stay invested. Apply for LAS with Shriram Financial Services.</t>
+          <t>Apply for the latest IPOs across NSE &amp; BSE and invest in companies as they debut on the stock market with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>/loan-against-shares</t>
+          <t>/ipo</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/loan-against-shares</t>
+          <t>https://thisisshon.github.io/ipo</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -1223,22 +1223,22 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Margin Trading Facility (MTF) | Shriram Financial Services</t>
+          <t>Loan Against Mutual Funds | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Get up to 4x buying power with Margin Trading Facility (MTF) from Shriram Financial Services - no overnight square-off, 700+ eligible stocks.</t>
+          <t>Get instant loans against your mutual fund holdings without redeeming investments. Quick, collateral-based LAMF from Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>/mtf</t>
+          <t>/loan-against-mutual-fund</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/mtf</t>
+          <t>https://thisisshon.github.io/loan-against-mutual-fund</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
@@ -1258,22 +1258,22 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Invest in Mutual Funds Online | Shriram Financial Services</t>
+          <t>Loan Against Shares (LAS) | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Compare 3,000+ mutual funds and invest in Regular and Direct Plans. Start a SIP from Rs 100/month with Shriram Financial Services.</t>
+          <t>Borrow against your equity portfolio at competitive interest rates while your shares stay invested. Apply for LAS with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>/mutual-funds</t>
+          <t>/loan-against-shares</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/mutual-funds</t>
+          <t>https://thisisshon.github.io/loan-against-shares</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -1293,22 +1293,22 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>New Fund Offer (NFO) Investing | Shriram Financial Services</t>
+          <t>Margin Trading Facility (MTF) | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Get first-mover advantage on newly launched mutual fund schemes at initial NAV pricing. Explore active NFOs with Shriram Financial Services.</t>
+          <t>Get up to 4x buying power with Margin Trading Facility (MTF) from Shriram Financial Services - no overnight square-off, 700+ eligible stocks.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>/nfo</t>
+          <t>/mtf</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/nfo</t>
+          <t>https://thisisshon.github.io/mtf</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
@@ -1328,22 +1328,22 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>National Pension Scheme (NPS) | Shriram Financial Services</t>
+          <t>Invest in Mutual Funds Online | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Build a tax-efficient retirement corpus with the government-backed National Pension Scheme. Save up to Rs 2 lakh in tax with Shriram.</t>
+          <t>Compare 3,000+ mutual funds and invest in Regular and Direct Plans. Start a SIP from Rs 100/month with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>/nps</t>
+          <t>/mutual-funds</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/nps</t>
+          <t>https://thisisshon.github.io/mutual-funds</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -1363,22 +1363,22 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Investment Products &amp; Trading | Shriram Financial Services</t>
+          <t>New Fund Offer (NFO) Investing | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Explore equity, derivatives, mutual funds, IPO, NPS, ETF, bonds &amp; Loan Against Mutual Fund - all investment products from Shriram Financial Services in one place.</t>
+          <t>Get first-mover advantage on newly launched mutual fund schemes at initial NAV pricing. Explore active NFOs with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>/products</t>
+          <t>/nfo</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/products</t>
+          <t>https://thisisshon.github.io/nfo</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1393,27 +1393,27 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Fundamental Research Reports | Shriram Financial Services</t>
+          <t>National Pension Scheme (NPS) | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Access in-depth company analysis, financial modelling and valuation reports to assess a stock's true worth with Shriram Financial Services.</t>
+          <t>Build a tax-efficient retirement corpus with the government-backed National Pension Scheme. Save up to Rs 2 lakh in tax with Shriram.</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>/fundamental-analysis</t>
+          <t>/nps</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/fundamental-analysis</t>
+          <t>https://thisisshon.github.io/nps</t>
         </is>
       </c>
       <c r="G27" s="11" t="inlineStr">
@@ -1428,27 +1428,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Products</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Mutual Fund Research &amp; Picks | Shriram Financial Services</t>
+          <t>Investment Products &amp; Trading | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Discover mutual fund research and expert fund picks to build a well-diversified portfolio with Shriram Financial Services.</t>
+          <t>Explore equity, derivatives, mutual funds, IPO, NPS, ETF, bonds &amp; Loan Against Mutual Fund - all investment products from Shriram Financial Services in one place.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>/mutual-fund-analysis</t>
+          <t>/products</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/mutual-fund-analysis</t>
+          <t>https://thisisshon.github.io/products</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -1468,22 +1468,22 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Stock Market Research Centre | Shriram Financial Services</t>
+          <t>Fundamental Research Reports | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Access technical, fundamental and mutual fund research to make informed investing decisions with SEBI-registered Shriram Financial Services.</t>
+          <t>Access in-depth company analysis, financial modelling and valuation reports to assess a stock's true worth with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>/research-hub</t>
+          <t>/fundamental-analysis</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/research-hub</t>
+          <t>https://thisisshon.github.io/fundamental-analysis</t>
         </is>
       </c>
       <c r="G29" s="11" t="inlineStr">
@@ -1503,22 +1503,22 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Technical Stock Research | Shriram Financial Services</t>
+          <t>Mutual Fund Research &amp; Picks | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Get technical research, chart patterns and trading ideas to time your entries and exits with Shriram Financial Services.</t>
+          <t>Discover mutual fund research and expert fund picks to build a well-diversified portfolio with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>/technical-analysis</t>
+          <t>/mutual-fund-analysis</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/technical-analysis</t>
+          <t>https://thisisshon.github.io/mutual-fund-analysis</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -1533,27 +1533,27 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Calculators</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Calculators | Shriram Financial Services</t>
+          <t>Stock Market Research Centre | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>Free financial calculators from Shriram - SIP, lumpsum, SWP, fixed deposit and NPS. Plan investments and estimate returns instantly, no sign-up.</t>
+          <t>Access technical, fundamental and mutual fund research to make informed investing decisions with SEBI-registered Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>/calculators</t>
+          <t>/research-hub</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/calculators</t>
+          <t>https://thisisshon.github.io/research-hub</t>
         </is>
       </c>
       <c r="G31" s="11" t="inlineStr">
@@ -1568,27 +1568,27 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Calculators</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Fixed Deposit Calculator | Shriram Financial Services</t>
+          <t>Technical Stock Research | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Calculate your fixed deposit maturity amount and interest earned instantly with the free FD calculator from Shriram Financial Services.</t>
+          <t>Get technical research, chart patterns and trading ideas to time your entries and exits with Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>/fd-calculator</t>
+          <t>/technical-analysis</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/fd-calculator</t>
+          <t>https://thisisshon.github.io/technical-analysis</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -1608,22 +1608,22 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Lumpsum Calculator Online | Shriram Financial Services</t>
+          <t>Calculators | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Estimate the future value of a one-time mutual fund investment with the free lumpsum calculator from Shriram Financial Services. Try it now.</t>
+          <t>Free financial calculators from Shriram - SIP, lumpsum, SWP, fixed deposit and NPS. Plan investments and estimate returns instantly, no sign-up.</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>/lumpsum-calculator</t>
+          <t>/calculators</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/lumpsum-calculator</t>
+          <t>https://thisisshon.github.io/calculators</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -1643,22 +1643,22 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>NPS Calculator - Pension | Shriram Financial Services</t>
+          <t>Fixed Deposit Calculator | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Estimate your NPS retirement corpus and monthly pension amount with the free NPS calculator from Shriram Financial Services. Plan today.</t>
+          <t>Calculate your fixed deposit maturity amount and interest earned instantly with the free FD calculator from Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>/nps-calculator</t>
+          <t>/fd-calculator</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/nps-calculator</t>
+          <t>https://thisisshon.github.io/fd-calculator</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -1678,22 +1678,22 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>SIP Calculator Online | Shriram Financial Services</t>
+          <t>Lumpsum Calculator Online | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Use the free SIP calculator from Shriram Financial Services to estimate your mutual fund returns based on amount, tenure and expected rate.</t>
+          <t>Estimate the future value of a one-time mutual fund investment with the free lumpsum calculator from Shriram Financial Services. Try it now.</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>/sip-calculator</t>
+          <t>/lumpsum-calculator</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/sip-calculator</t>
+          <t>https://thisisshon.github.io/lumpsum-calculator</t>
         </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
@@ -1713,22 +1713,22 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>SWP Calculator - Withdrawal | Shriram Financial Services</t>
+          <t>NPS Calculator - Pension | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Plan your regular mutual fund withdrawals and estimate your remaining corpus with the free SWP calculator from Shriram Financial Services.</t>
+          <t>Estimate your NPS retirement corpus and monthly pension amount with the free NPS calculator from Shriram Financial Services. Plan today.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>/swp-calculator</t>
+          <t>/nps-calculator</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/swp-calculator</t>
+          <t>https://thisisshon.github.io/nps-calculator</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -1743,27 +1743,27 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Calculators</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Contact &amp; Customer Support | Shriram Financial Services</t>
+          <t>SIP Calculator Online | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Get in touch with Shriram Financial Services for account help, trading queries or a free discovery call with a dedicated wealth advisor.</t>
+          <t>Use the free SIP calculator from Shriram Financial Services to estimate your mutual fund returns based on amount, tenure and expected rate.</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>/contact-us</t>
+          <t>/sip-calculator</t>
         </is>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/contact-us</t>
+          <t>https://thisisshon.github.io/sip-calculator</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -1778,27 +1778,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Calculators</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Grievance Redressal Process | Shriram Financial Services</t>
+          <t>SWP Calculator - Withdrawal | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Learn how to raise and track a complaint through the Grievance Redressal Mechanism of Shriram Financial Services.</t>
+          <t>Plan your regular mutual fund withdrawals and estimate your remaining corpus with the free SWP calculator from Shriram Financial Services.</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>/grievance-redressal</t>
+          <t>/swp-calculator</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/grievance-redressal</t>
+          <t>https://thisisshon.github.io/swp-calculator</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -1813,27 +1813,27 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Legal &amp; Compliance</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Privacy Policy | Shriram Financial Services</t>
+          <t>Contact &amp; Customer Support | Shriram Financial Services</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Read the Privacy Policy of Shriram Financial Services to understand how your personal and financial data is collected, used and protected.</t>
+          <t>Get in touch with Shriram Financial Services for account help, trading queries or a free discovery call with a dedicated wealth advisor.</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>/privacy-policy</t>
+          <t>/contact-us</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>https://thisisshon.github.io/privacy-policy</t>
+          <t>https://thisisshon.github.io/contact-us</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
@@ -1848,275 +1848,380 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Grievance Redressal Process | Shriram Financial Services</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Learn how to raise and track a complaint through the Grievance Redressal Mechanism of Shriram Financial Services.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>/grievance-redressal</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>https://thisisshon.github.io/grievance-redressal</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>FAQs - Answers on Every Product | Shriram Financial Services</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Browse 170+ frequently asked questions across Shriram's trading, investing, new-issue and loan-against-securities products, or ask our on-page FAQ assistant.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>/faqs</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>https://thisisshon.github.io/faqs</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
           <t>Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Privacy Policy | Shriram Financial Services</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Read the Privacy Policy of Shriram Financial Services to understand how your personal and financial data is collected, used and protected.</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>/privacy-policy</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>https://thisisshon.github.io/privacy-policy</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Legal &amp; Compliance</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Regulatory Info &amp; Compliance | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>View SEBI registration numbers, exchange memberships and compliance disclosures for Shriram Financial Services.</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>/regulatorydocuments</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/regulatorydocuments</t>
         </is>
       </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>Investor Charter - Rights | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D44" s="9" t="inlineStr">
         <is>
           <t>Read the SEBI-mandated Investor Charter outlining your rights, responsibilities and grievance process with Shriram Financial Services.</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>/regulatorydocuments/investor-charter</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr">
+      <c r="F44" s="10" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/regulatorydocuments/investor-charter</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
-        <v>39</v>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Mandatory Member Details | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>All mandatory disclosures, investor rights, grievance mechanisms and compliance documents - in one place. View online or download as PDF.</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>/regulatorydocuments/mandatory-member-details</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/regulatorydocuments/mandatory-member-details</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>Terms &amp; Conditions | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D46" s="9" t="inlineStr">
         <is>
           <t>Read the Terms &amp; Conditions governing the use of Shriram Financial Services' trading, investment &amp; related services.</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t>/terms-and-conditions</t>
         </is>
       </c>
-      <c r="F43" s="10" t="inlineStr">
+      <c r="F46" s="10" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/terms-and-conditions</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Legal &amp; Compliance</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>Terms of Use - Purse App | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>The Terms of Use for Purse App by Shriram Financial Services before using its trading &amp; investment features.</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>/terms-of-use-purse</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/terms-of-use-purse</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="n">
-        <v>42</v>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>Design System - Documentation Hub | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
         <is>
           <t>Internal design-system documentation for Shriram Financial Services: the honest as-built style inventory of the legacy site, and the consolidated token system rendered live from styles.css for the Figma round-trip.</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>/designsystem</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
+      <c r="F48" s="10" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/designsystem</t>
         </is>
       </c>
-      <c r="G45" s="12" t="inlineStr">
+      <c r="G48" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B46" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Design System - What Is Used (Legacy Inventory) | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>The honest as-built style inventory of the legacy Shriram site: ~150 colors grouped by near-duplicate cluster, the two-stylesheet fork, and the off-scale type / off-grid spacing / gradient recipes the token system resolves.</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>/designsystem/current</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/designsystem/current</t>
         </is>
       </c>
-      <c r="G46" s="13" t="inlineStr">
+      <c r="G49" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="8" t="n">
-        <v>44</v>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>Design System - What Is Suggested (Live Token Reference) | Shriram Financial Services</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D50" s="9" t="inlineStr">
         <is>
           <t>The consolidated Shriram design system rendered live from styles.css: primitive → semantic → component colour tokens, the type scale, 8px spacing + radii, shadows, motion and a component gallery - structured to map 1:1 onto Figma variables.</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E50" s="8" t="inlineStr">
         <is>
           <t>/designsystem/proposed</t>
         </is>
       </c>
-      <c r="F47" s="10" t="inlineStr">
+      <c r="F50" s="10" t="inlineStr">
         <is>
           <t>https://thisisshon.github.io/designsystem/proposed</t>
         </is>
       </c>
-      <c r="G47" s="12" t="inlineStr">
+      <c r="G50" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>